<commit_message>
docs: address Purview label review findings
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/compliance-officer-checklist.xlsx
+++ b/assessment/templates/compliance-officer-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Compliance Officer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance Officer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Compliance Officer'!$A$4:$I$26</definedName>
@@ -715,7 +715,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Sensitivity-label taxonomy with Copilot content classification mapping; Auto-labeling policy configuration and coverage report; Label usage report from Activity Explorer for the last 30 days; Evidence of label propagation to Copilot-generated outputs</t>
+          <t>Sensitivity-label taxonomy with Copilot content classification mapping; Auto-labeling policy configuration plus Coverage by simulation context or Labeled items review evidence; Activity Explorer sensitivity-label activity for the last 30 days; Evidence of label propagation to Copilot-generated outputs</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: re-verify Purview and Defender governance controls
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/compliance-officer-checklist.xlsx
+++ b/assessment/templates/compliance-officer-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Compliance Officer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance Officer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Compliance Officer'!$A$4:$I$26</definedName>
@@ -754,7 +754,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Insider Risk policy configuration including Copilot indicators; Alert triage cadence and escalation path documentation; Recent alert review log (last 30 days); Integration with HR/legal escalation workflows</t>
+          <t>Insider Risk policy configuration including Generative AI apps indicators and any Risky AI usage indicators; Alert triage cadence and escalation path documentation; Recent alert review log (last 30 days), including Risky Agents coverage where applicable; Integration with HR/legal escalation workflows</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: refresh Purview sensitivity label guidance (#566)
Part of the documentation freshness program.
</commit_message>
<xml_diff>
--- a/assessment/templates/compliance-officer-checklist.xlsx
+++ b/assessment/templates/compliance-officer-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Compliance Officer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance Officer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Compliance Officer'!$A$4:$I$26</definedName>
@@ -715,7 +715,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Sensitivity-label taxonomy with Copilot content classification mapping; Auto-labeling policy configuration and coverage report; Label usage report from Activity Explorer for the last 30 days; Evidence of label propagation to Copilot-generated outputs</t>
+          <t>Sensitivity-label taxonomy with Copilot content classification mapping; Auto-labeling policy configuration plus Coverage by simulation context or Labeled items review evidence; Activity Explorer sensitivity-label activity for the last 30 days; Evidence of label propagation to Copilot-generated outputs</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>

</xml_diff>